<commit_message>
minor changes in gm-selection input
</commit_message>
<xml_diff>
--- a/HazardAnalysis/gm-selection/2020_NBC_MyCopy_new-main/GMSelection_NGA_KiK_mixed/Inputs_IS2026.xlsx
+++ b/HazardAnalysis/gm-selection/2020_NBC_MyCopy_new-main/GMSelection_NGA_KiK_mixed/Inputs_IS2026.xlsx
@@ -1,24 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\OpenSees_PracticeExamples\ida-spo-msa\HazardAnalysis\gm-selection\2020_NBC_MyCopy_new-main\GMSelection_NGA_KiK_mixed\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\psb\Downloads\GitHub\ida-spo-msa\HazardAnalysis\gm-selection\2020_NBC_MyCopy_new-main\GMSelection_NGA_KiK_mixed\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDC79725-36A3-46DE-96A7-ECF1ADC6CBD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="11775"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
     <sheet name="fixedInfo" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -353,7 +365,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -655,7 +667,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -666,9 +678,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -693,7 +702,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -702,7 +711,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
@@ -749,12 +758,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -773,10 +776,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -813,10 +816,10 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -834,7 +837,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -855,16 +858,10 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1186,7 +1183,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L250"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1208,306 +1205,304 @@
       <c r="A2" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="I2" s="63"/>
+      <c r="I2" s="60"/>
     </row>
     <row r="3" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I3" s="64" t="s">
+      <c r="I3" s="61" t="s">
         <v>49</v>
       </c>
-      <c r="J3" s="59"/>
+      <c r="J3" s="56"/>
     </row>
     <row r="4" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="69" t="s">
+      <c r="F4" s="66" t="s">
         <v>55</v>
       </c>
-      <c r="G4" s="70"/>
-      <c r="I4" s="60" t="s">
+      <c r="G4" s="67"/>
+      <c r="I4" s="57" t="s">
         <v>30</v>
       </c>
-      <c r="J4" s="61">
+      <c r="J4" s="58">
         <v>1.5</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="F5" s="71" t="s">
+      <c r="F5" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="G5" s="72" t="s">
+      <c r="G5" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="I5" s="56" t="s">
+      <c r="I5" s="53" t="s">
         <v>31</v>
       </c>
-      <c r="J5" s="47">
+      <c r="J5" s="44">
         <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="4">
         <v>91.77</v>
       </c>
-      <c r="F6" s="22">
+      <c r="F6" s="21">
         <f t="shared" ref="F6" si="0">MIN(0.15*$C$9, $C$10)</f>
         <v>0.1065</v>
       </c>
-      <c r="G6" s="23">
+      <c r="G6" s="22">
         <f t="shared" ref="G6" si="1">MAX(2*$C$9, 1.5)</f>
         <v>1.5</v>
       </c>
-      <c r="I6" s="55" t="s">
+      <c r="I6" s="52" t="s">
         <v>32</v>
       </c>
-      <c r="J6" s="47">
-        <v>300</v>
+      <c r="J6" s="44">
+        <v>400</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="73">
+      <c r="C7" s="68">
         <v>26.17</v>
       </c>
-      <c r="I7" s="62" t="s">
+      <c r="I7" s="59" t="s">
         <v>33</v>
       </c>
-      <c r="J7" s="57">
-        <v>800</v>
+      <c r="J7" s="54">
+        <v>1500</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="5">
-        <v>500</v>
+      <c r="C8" s="4">
+        <v>760</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="I8" s="65" t="s">
+      <c r="I8" s="62" t="s">
         <v>48</v>
       </c>
-      <c r="J8" s="66" t="s">
+      <c r="J8" s="63" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="5">
+      <c r="C9" s="4">
         <v>0.71</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="I9" s="67" t="s">
+      <c r="I9" s="64" t="s">
         <v>47</v>
       </c>
-      <c r="J9" s="68">
+      <c r="J9" s="65">
         <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="5">
+      <c r="C10" s="4">
         <v>0.25</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E10" s="46" t="s">
+      <c r="E10" s="43" t="s">
         <v>7</v>
       </c>
-      <c r="F10" s="46"/>
+      <c r="F10" s="43"/>
     </row>
     <row r="11" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="5">
+      <c r="C11" s="4">
         <v>0.54</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="E11" s="46" t="s">
+      <c r="E11" s="43" t="s">
         <v>37</v>
       </c>
-      <c r="F11" s="46"/>
-    </row>
-    <row r="12" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="4"/>
-    </row>
+      <c r="F11" s="43"/>
+    </row>
+    <row r="12" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="13" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:12" s="5" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="14"/>
-      <c r="B14" s="19" t="s">
+    <row r="14" spans="1:12" s="4" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="13"/>
+      <c r="B14" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="20" t="s">
+      <c r="C14" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="D14" s="20" t="s">
+      <c r="D14" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="E14" s="48" t="s">
+      <c r="E14" s="45" t="s">
         <v>41</v>
       </c>
-      <c r="F14" s="31" t="s">
+      <c r="F14" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="G14" s="30" t="s">
+      <c r="G14" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="H14" s="31"/>
-      <c r="I14" s="27" t="s">
+      <c r="H14" s="30"/>
+      <c r="I14" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="J14" s="28"/>
-      <c r="K14" s="40" t="s">
+      <c r="J14" s="27"/>
+      <c r="K14" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="L14" s="28" t="s">
+      <c r="L14" s="27" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="35"/>
-      <c r="B15" s="37"/>
-      <c r="C15" s="36"/>
-      <c r="D15" s="45" t="s">
+    <row r="15" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="32"/>
+      <c r="B15" s="34"/>
+      <c r="C15" s="33"/>
+      <c r="D15" s="42" t="s">
         <v>46</v>
       </c>
-      <c r="E15" s="49"/>
-      <c r="F15" s="50"/>
-      <c r="G15" s="41" t="s">
+      <c r="E15" s="46"/>
+      <c r="F15" s="47"/>
+      <c r="G15" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="H15" s="42"/>
-      <c r="I15" s="43" t="s">
+      <c r="H15" s="39"/>
+      <c r="I15" s="40" t="s">
         <v>8</v>
       </c>
-      <c r="J15" s="44" t="s">
+      <c r="J15" s="41" t="s">
         <v>8</v>
       </c>
-      <c r="K15" s="43" t="s">
+      <c r="K15" s="40" t="s">
         <v>8</v>
       </c>
-      <c r="L15" s="44" t="s">
+      <c r="L15" s="41" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="18" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
-      <c r="B16" s="6"/>
-      <c r="C16" s="58">
+      <c r="B16" s="5"/>
+      <c r="C16" s="55">
         <f>SUM(C17:C18)</f>
+        <v>30</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="E16" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="F16" s="28" t="s">
+        <v>43</v>
+      </c>
+      <c r="G16" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="H16" s="28" t="s">
+        <v>15</v>
+      </c>
+      <c r="I16" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="J16" s="28" t="s">
+        <v>18</v>
+      </c>
+      <c r="K16" s="31" t="s">
+        <v>8</v>
+      </c>
+      <c r="L16" s="20" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C17" s="10">
+        <v>30</v>
+      </c>
+      <c r="D17" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="D16" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="E16" s="32" t="s">
-        <v>42</v>
-      </c>
-      <c r="F16" s="33" t="s">
-        <v>43</v>
-      </c>
-      <c r="G16" s="32" t="s">
-        <v>14</v>
-      </c>
-      <c r="H16" s="33" t="s">
-        <v>15</v>
-      </c>
-      <c r="I16" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="J16" s="29" t="s">
-        <v>18</v>
-      </c>
-      <c r="K16" s="34" t="s">
-        <v>8</v>
-      </c>
-      <c r="L16" s="21" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="C17" s="11">
-        <v>40</v>
-      </c>
-      <c r="D17" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="E17" s="51">
+      <c r="E17" s="48">
         <f t="shared" ref="E17" si="2">$C$9</f>
         <v>0.71</v>
       </c>
-      <c r="F17" s="53">
+      <c r="F17" s="50">
         <f t="shared" ref="F17" si="3">$C$11</f>
         <v>0.54</v>
       </c>
-      <c r="G17" s="34">
+      <c r="G17" s="31">
         <f t="shared" ref="G17" si="4">MIN(0.15*$C$9, $C$10)</f>
         <v>0.1065</v>
       </c>
-      <c r="H17" s="21">
+      <c r="H17" s="20">
         <f t="shared" ref="H17" si="5">MAX(2*$C$9, 1.5)</f>
         <v>1.5</v>
       </c>
-      <c r="I17" s="54">
+      <c r="I17" s="51">
         <v>7</v>
       </c>
-      <c r="J17" s="21">
+      <c r="J17" s="20">
         <v>25</v>
       </c>
-      <c r="K17" s="34" t="s">
+      <c r="K17" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="L17" s="38" t="s">
+      <c r="L17" s="35" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="12" t="s">
+      <c r="B18" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="52"/>
-      <c r="F18" s="39"/>
-      <c r="G18" s="22"/>
-      <c r="H18" s="23"/>
-      <c r="I18" s="25"/>
-      <c r="J18" s="26"/>
-      <c r="K18" s="22"/>
-      <c r="L18" s="39"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="49"/>
+      <c r="F18" s="36"/>
+      <c r="G18" s="21"/>
+      <c r="H18" s="22"/>
+      <c r="I18" s="24"/>
+      <c r="J18" s="25"/>
+      <c r="K18" s="21"/>
+      <c r="L18" s="36"/>
     </row>
     <row r="19" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C19" s="9"/>
+      <c r="C19" s="8"/>
     </row>
     <row r="20" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
@@ -1523,7 +1518,7 @@
     <row r="25" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="27" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="8"/>
+      <c r="B27" s="7"/>
     </row>
     <row r="28" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="29" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1750,19 +1745,19 @@
     <row r="250" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G15">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G15" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"NBCC (Single Building), Manual (Deaggregation-Based)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J8">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J8" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Yes, No"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D17:D18">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D17:D18" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"NGA_W2, KiK_NET"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L17:L18">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L17:L18" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"Strike-slip, Normal, Reverse, Unknown"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B17:B18">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B17:B18" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Crustal,In-slab,Interface/Subduction,Any"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1771,7 +1766,7 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" showInputMessage="1" showErrorMessage="1">
+        <x14:dataValidation type="list" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000005000000}">
           <x14:formula1>
             <xm:f>fixedInfo!$D$3:$D$22</xm:f>
           </x14:formula1>
@@ -1784,7 +1779,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="D1:D31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1793,107 +1788,107 @@
   <sheetData>
     <row r="1" spans="4:4" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="4:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="14" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="3" spans="4:4" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D3" s="16" t="s">
+      <c r="D3" s="15" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="4" spans="4:4" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D4" s="17" t="s">
+      <c r="D4" s="16" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="5" spans="4:4" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D5" s="17" t="s">
+      <c r="D5" s="16" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="6" spans="4:4" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D6" s="17" t="s">
+      <c r="D6" s="16" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="7" spans="4:4" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D7" s="17" t="s">
+      <c r="D7" s="16" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="8" spans="4:4" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D8" s="17" t="s">
+      <c r="D8" s="16" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="9" spans="4:4" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D9" s="17" t="s">
+      <c r="D9" s="16" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="10" spans="4:4" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D10" s="17" t="s">
+      <c r="D10" s="16" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="11" spans="4:4" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D11" s="17" t="s">
+      <c r="D11" s="16" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="12" spans="4:4" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D12" s="17" t="s">
+      <c r="D12" s="16" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="13" spans="4:4" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D13" s="17" t="s">
+      <c r="D13" s="16" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="14" spans="4:4" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D14" s="17" t="s">
+      <c r="D14" s="16" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="15" spans="4:4" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D15" s="17" t="s">
+      <c r="D15" s="16" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="16" spans="4:4" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D16" s="17" t="s">
+      <c r="D16" s="16" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="17" spans="4:4" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D17" s="17" t="s">
+      <c r="D17" s="16" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="18" spans="4:4" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D18" s="17" t="s">
+      <c r="D18" s="16" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="19" spans="4:4" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D19" s="17" t="s">
+      <c r="D19" s="16" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="20" spans="4:4" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D20" s="17" t="s">
+      <c r="D20" s="16" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="21" spans="4:4" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D21" s="17" t="s">
+      <c r="D21" s="16" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="22" spans="4:4" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D22" s="18"/>
+      <c r="D22" s="17"/>
     </row>
     <row r="23" spans="4:4" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="24" spans="4:4" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
minor update in calling ASK14, CY14
</commit_message>
<xml_diff>
--- a/HazardAnalysis/gm-selection/2020_NBC_MyCopy_new-main/GMSelection_NGA_KiK_mixed/Inputs_IS2026.xlsx
+++ b/HazardAnalysis/gm-selection/2020_NBC_MyCopy_new-main/GMSelection_NGA_KiK_mixed/Inputs_IS2026.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\OpenSees_PracticeExamples\ida-spo-msa\HazardAnalysis\gm-selection\2020_NBC_MyCopy_new-main\GMSelection_NGA_KiK_mixed\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\psb\Downloads\GitHub\ida-spo-msa\HazardAnalysis\gm-selection\2020_NBC_MyCopy_new-main\GMSelection_NGA_KiK_mixed\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20FEC310-2A7D-4393-A2BD-A8B26895DDAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
     <sheet name="fixedInfo" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -370,7 +371,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1221,7 +1222,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L250"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1782,20 +1783,20 @@
     <row r="249" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="250" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <dataValidations disablePrompts="1" count="5">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G15">
+  <dataValidations count="5">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G15" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"NBCC (Single Building), Manual (Deaggregation-Based)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J8">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J8" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Yes, No"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D17:D18">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D17:D18" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"NGA_W2, KiK_NET"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L17:L18">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L17:L18" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"Strike-slip, Normal, Reverse, Unknown"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B17:B18">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B17:B18" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Crustal,In-slab,Interface/Subduction,Any"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1803,8 +1804,8 @@
   <pageSetup orientation="portrait" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="1">
-        <x14:dataValidation type="list" showInputMessage="1" showErrorMessage="1">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000005000000}">
           <x14:formula1>
             <xm:f>fixedInfo!$D$3:$D$22</xm:f>
           </x14:formula1>
@@ -1817,7 +1818,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="D1:D31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>